<commit_message>
Refine historical typography and workbook previews
</commit_message>
<xml_diff>
--- a/results/江右游日记_二十三日_步驟一_地名抽取.xlsx
+++ b/results/江右游日记_二十三日_步驟一_地名抽取.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步驟一｜二十三日經過地名抽取" sheetId="1" r:id="R431e0a4821c64dfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江右游日记_篩除" sheetId="2" r:id="Re7b919abcbae4567"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="步驟一｜二十三日經過地名抽取" sheetId="1" r:id="R065a309a5de34328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="江右游日记_篩除" sheetId="2" r:id="R044c814e067841c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -624,8 +624,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Day23Step1PassedRecords" displayName="Day23Step1PassedRecords" ref="A7:M32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A7:M32"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="Day23Step1PassedRecords" displayName="Day23Step1PassedRecords" ref="A3:M28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A3:M28"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="序號"/>
     <x:tableColumn id="2" name="日期"/>
@@ -893,1030 +893,1372 @@
       <x:c r="K1" s="139"/>
       <x:c r="L1" s="139"/>
       <x:c r="M1" s="139"/>
-    </x:row>
-    <x:row r="2" ht="22.5" customHeight="1">
-      <x:c r="A2" s="143" t="str">
-        <x:v>篩選結果｜25 筆</x:v>
-      </x:c>
-      <x:c r="B2" s="143"/>
-      <x:c r="C2" s="143"/>
-      <x:c r="D2" s="143"/>
-      <x:c r="E2" s="143"/>
-      <x:c r="F2" s="143"/>
-      <x:c r="G2" s="143"/>
-      <x:c r="H2" s="143"/>
-      <x:c r="I2" s="143"/>
-      <x:c r="J2" s="143"/>
-      <x:c r="K2" s="143"/>
-      <x:c r="L2" s="143"/>
-      <x:c r="M2" s="143"/>
-    </x:row>
-    <x:row r="3" ht="43.5" customHeight="1">
-      <x:c r="A3" s="147" t="str">
-        <x:v>只保留二十三日且行程＝經過的 25 筆；按原文出現次序保留重複地名。篩除項目另見「江右游日记_篩除」worksheet。</x:v>
-      </x:c>
-      <x:c r="B3" s="147"/>
-      <x:c r="C3" s="147"/>
-      <x:c r="D3" s="147"/>
-      <x:c r="E3" s="147"/>
-      <x:c r="F3" s="147"/>
-      <x:c r="G3" s="147"/>
-      <x:c r="H3" s="147"/>
-      <x:c r="I3" s="147"/>
-      <x:c r="J3" s="147"/>
-      <x:c r="K3" s="147"/>
-      <x:c r="L3" s="147"/>
-      <x:c r="M3" s="147"/>
-    </x:row>
-    <x:row r="4" ht="18.75" customHeight="1">
-      <x:c r="A4" s="151" t="str">
-        <x:v>Prompt｜本步驟獨立操作指令</x:v>
-      </x:c>
-      <x:c r="B4" s="151"/>
-      <x:c r="C4" s="151"/>
-      <x:c r="D4" s="151"/>
-      <x:c r="E4" s="151"/>
-      <x:c r="F4" s="151"/>
-      <x:c r="G4" s="151"/>
-      <x:c r="H4" s="151"/>
-      <x:c r="I4" s="151"/>
-      <x:c r="J4" s="151"/>
-      <x:c r="K4" s="151"/>
-      <x:c r="L4" s="151"/>
-      <x:c r="M4" s="151"/>
-    </x:row>
-    <x:row r="5" ht="75" customHeight="1">
-      <x:c r="A5" s="147" t="str">
-        <x:v>請只處理《江右游日記》二十三日段落，按出現次序抽取具名地理實體；輸出只保留行程欄等於「經過」的紀錄。輸出序號、日期、地名、類別、細分類、行程及原文；重複出現的地名保留每次紀錄。橋、城門、驛站、碼頭、私人住所、建築內部小物及修辭方向詞，另列入篩除表，不得當作正式地標。</x:v>
-      </x:c>
-      <x:c r="B5" s="147"/>
-      <x:c r="C5" s="147"/>
-      <x:c r="D5" s="147"/>
-      <x:c r="E5" s="147"/>
-      <x:c r="F5" s="147"/>
-      <x:c r="G5" s="147"/>
-      <x:c r="H5" s="147"/>
-      <x:c r="I5" s="147"/>
-      <x:c r="J5" s="147"/>
-      <x:c r="K5" s="147"/>
-      <x:c r="L5" s="147"/>
-      <x:c r="M5" s="147"/>
+      <x:c r="AA1"/>
+      <x:c r="AB1"/>
+      <x:c r="AC1"/>
+      <x:c r="AD1"/>
+      <x:c r="AE1"/>
+      <x:c r="AF1"/>
+      <x:c r="AG1"/>
+      <x:c r="AH1"/>
+      <x:c r="AI1"/>
+      <x:c r="AJ1"/>
+      <x:c r="AK1"/>
+      <x:c r="AL1"/>
+      <x:c r="AM1"/>
+    </x:row>
+    <x:row r="2" ht="54" customHeight="1">
+      <x:c r="A2"/>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
+      <x:c r="F2"/>
+      <x:c r="G2"/>
+      <x:c r="H2"/>
+      <x:c r="I2"/>
+      <x:c r="J2"/>
+      <x:c r="K2"/>
+      <x:c r="L2"/>
+      <x:c r="M2"/>
+      <x:c r="AA2"/>
+      <x:c r="AB2"/>
+      <x:c r="AC2"/>
+      <x:c r="AD2"/>
+      <x:c r="AE2"/>
+      <x:c r="AF2"/>
+      <x:c r="AG2"/>
+      <x:c r="AH2"/>
+      <x:c r="AI2"/>
+      <x:c r="AJ2"/>
+      <x:c r="AK2"/>
+      <x:c r="AL2"/>
+      <x:c r="AM2"/>
+    </x:row>
+    <x:row r="3" ht="36" customHeight="1">
+      <x:c r="A3" t="str">
+        <x:v>序號</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>地名</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>類別</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>細分類</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>行程</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>原文</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>第一地方志配對</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>地方志原句</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
+        <x:v>第二地方志</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>record_level</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>gis_decision</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>判斷理由</x:v>
+      </x:c>
+      <x:c r="AA3"/>
+      <x:c r="AB3"/>
+      <x:c r="AC3"/>
+      <x:c r="AD3"/>
+      <x:c r="AE3"/>
+      <x:c r="AF3"/>
+      <x:c r="AG3"/>
+      <x:c r="AH3"/>
+      <x:c r="AI3"/>
+      <x:c r="AJ3"/>
+      <x:c r="AK3"/>
+      <x:c r="AL3"/>
+      <x:c r="AM3"/>
+    </x:row>
+    <x:row r="4" ht="54" customHeight="1">
+      <x:c r="A4" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>贵溪城</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>行政區</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>城市／城</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>晨起，渡大溪之北，复西向行，八里，将至贵溪城，忽见溪南一桥门架空，以为城门与卷梁皆无此高跨之理。</x:v>
+      </x:c>
+      <x:c r="H4"/>
+      <x:c r="I4"/>
+      <x:c r="J4"/>
+      <x:c r="K4" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>貴溪城為縣城，作者將至，重要節點。</x:v>
+      </x:c>
+      <x:c r="AA4"/>
+      <x:c r="AB4"/>
+      <x:c r="AC4"/>
+      <x:c r="AD4"/>
+      <x:c r="AE4"/>
+      <x:c r="AF4"/>
+      <x:c r="AG4"/>
+      <x:c r="AH4"/>
+      <x:c r="AI4"/>
+      <x:c r="AJ4"/>
+      <x:c r="AK4"/>
+      <x:c r="AL4"/>
+      <x:c r="AM4"/>
+    </x:row>
+    <x:row r="5" ht="54" customHeight="1">
+      <x:c r="A5" t="n">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>张真人墓</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>歷史遺址</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>墓葬／陵墓</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>于是南经张真人墓。</x:v>
+      </x:c>
+      <x:c r="H5"/>
+      <x:c r="I5"/>
+      <x:c r="J5"/>
+      <x:c r="K5" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>作者實際經過之墓葬（張真人墓），為具名地標</x:v>
+      </x:c>
+      <x:c r="AA5"/>
+      <x:c r="AB5"/>
+      <x:c r="AC5"/>
+      <x:c r="AD5"/>
+      <x:c r="AE5"/>
+      <x:c r="AF5"/>
+      <x:c r="AG5"/>
+      <x:c r="AH5"/>
+      <x:c r="AI5"/>
+      <x:c r="AJ5"/>
+      <x:c r="AK5"/>
+      <x:c r="AL5"/>
+      <x:c r="AM5"/>
     </x:row>
     <x:row r="6" ht="54" customHeight="1">
-      <x:c r="A6"/>
-      <x:c r="B6"/>
-      <x:c r="C6"/>
-      <x:c r="D6"/>
-      <x:c r="E6"/>
-      <x:c r="F6"/>
-      <x:c r="G6"/>
+      <x:c r="A6" t="n">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>五面峰</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>山峰</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>溪流直逼五面峰下。</x:v>
+      </x:c>
       <x:c r="H6"/>
       <x:c r="I6"/>
       <x:c r="J6"/>
-    </x:row>
-    <x:row r="7" ht="36" customHeight="1">
-      <x:c r="A7" s="155" t="str">
-        <x:v>序號</x:v>
-      </x:c>
-      <x:c r="B7" s="155" t="str">
-        <x:v>日期</x:v>
-      </x:c>
-      <x:c r="C7" s="155" t="str">
-        <x:v>地名</x:v>
-      </x:c>
-      <x:c r="D7" s="155" t="str">
-        <x:v>類別</x:v>
-      </x:c>
-      <x:c r="E7" s="155" t="str">
-        <x:v>細分類</x:v>
-      </x:c>
-      <x:c r="F7" s="155" t="str">
-        <x:v>行程</x:v>
-      </x:c>
-      <x:c r="G7" s="155" t="str">
-        <x:v>原文</x:v>
-      </x:c>
-      <x:c r="H7" s="155" t="str">
-        <x:v>第一地方志配對</x:v>
-      </x:c>
-      <x:c r="I7" s="155" t="str">
-        <x:v>地方志原句</x:v>
-      </x:c>
-      <x:c r="J7" s="155" t="str">
-        <x:v>第二地方志</x:v>
-      </x:c>
-      <x:c r="K7" s="155" t="str">
-        <x:v>record_level</x:v>
-      </x:c>
-      <x:c r="L7" s="155" t="str">
-        <x:v>gis_decision</x:v>
-      </x:c>
-      <x:c r="M7" s="155" t="str">
-        <x:v>判斷理由</x:v>
-      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>作者實際抵達之山峰，為穩定地理實體</x:v>
+      </x:c>
+      <x:c r="AA6"/>
+      <x:c r="AB6"/>
+      <x:c r="AC6"/>
+      <x:c r="AD6"/>
+      <x:c r="AE6"/>
+      <x:c r="AF6"/>
+      <x:c r="AG6"/>
+      <x:c r="AH6"/>
+      <x:c r="AI6"/>
+      <x:c r="AJ6"/>
+      <x:c r="AK6"/>
+      <x:c r="AL6"/>
+      <x:c r="AM6"/>
+    </x:row>
+    <x:row r="7" ht="54" customHeight="1">
+      <x:c r="A7" t="n">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>一线天</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>峽谷</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>余意南下者为一线天，西上者为五面峰也。</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>《弋阳县志》卷首〈龟峰图说〉｜識典古籍｜https://www.shidianguji.com/book/NLG312001072192/chapter/1ll4vbz35hwky</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>自此逾岭，双崖中裂，曰一线天。</x:v>
+      </x:c>
+      <x:c r="J7"/>
+      <x:c r="K7" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>作者實際遊覽之一線天，為重要自然景觀</x:v>
+      </x:c>
+      <x:c r="AA7"/>
+      <x:c r="AB7"/>
+      <x:c r="AC7"/>
+      <x:c r="AD7"/>
+      <x:c r="AE7"/>
+      <x:c r="AF7"/>
+      <x:c r="AG7"/>
+      <x:c r="AH7"/>
+      <x:c r="AI7"/>
+      <x:c r="AJ7"/>
+      <x:c r="AK7"/>
+      <x:c r="AL7"/>
+      <x:c r="AM7"/>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
-      <x:c r="A8" s="59" t="n">
-        <x:v>164</x:v>
-      </x:c>
-      <x:c r="B8" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C8" s="59" t="str">
-        <x:v>贵溪城</x:v>
-      </x:c>
-      <x:c r="D8" s="59" t="str">
+      <x:c r="A8" t="n">
+        <x:v>191</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>五面峰</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>山峰</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>余意南下者为一线天，西上者为五面峰也。</x:v>
+      </x:c>
+      <x:c r="H8"/>
+      <x:c r="I8"/>
+      <x:c r="J8"/>
+      <x:c r="K8" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L8" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M8" t="str">
+        <x:v>作者實際攀登之五面峰，為穩定地理實體</x:v>
+      </x:c>
+      <x:c r="AA8"/>
+      <x:c r="AB8"/>
+      <x:c r="AC8"/>
+      <x:c r="AD8"/>
+      <x:c r="AE8"/>
+      <x:c r="AF8"/>
+      <x:c r="AG8"/>
+      <x:c r="AH8"/>
+      <x:c r="AI8"/>
+      <x:c r="AJ8"/>
+      <x:c r="AK8"/>
+      <x:c r="AL8"/>
+      <x:c r="AM8"/>
+    </x:row>
+    <x:row r="9" ht="54" customHeight="1">
+      <x:c r="A9" t="n">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>西华</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>先跻峰，攀磴里许而至绝顶，则南瞰西华，东瞰夹壁，西瞰南溪，北瞰城邑，皆在指顾。</x:v>
+      </x:c>
+      <x:c r="H9"/>
+      <x:c r="I9"/>
+      <x:c r="J9"/>
+      <x:c r="K9" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L9" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M9" t="str">
+        <x:v>作者實際眺望之西華山，為穩定地理實體</x:v>
+      </x:c>
+      <x:c r="AA9"/>
+      <x:c r="AB9"/>
+      <x:c r="AC9"/>
+      <x:c r="AD9"/>
+      <x:c r="AE9"/>
+      <x:c r="AF9"/>
+      <x:c r="AG9"/>
+      <x:c r="AH9"/>
+      <x:c r="AI9"/>
+      <x:c r="AJ9"/>
+      <x:c r="AK9"/>
+      <x:c r="AL9"/>
+      <x:c r="AM9"/>
+    </x:row>
+    <x:row r="10" ht="54" customHeight="1">
+      <x:c r="A10" t="n">
+        <x:v>195</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>一线天</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>峽谷</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>复从前磴南下一线天，则两崖并夹而上，直南即从峰顶下剖者，是为直峡。</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>《弋阳县志》卷首〈龟峰图说〉｜識典古籍｜https://www.shidianguji.com/book/NLG312001072192/chapter/1ll4vbz35hwky</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>自此逾岭，双崖中裂，曰一线天。</x:v>
+      </x:c>
+      <x:c r="J10"/>
+      <x:c r="K10" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L10" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M10" t="str">
+        <x:v>一線天為作者親身經過的具名峽谷或岩隙景觀，屬地理實體，非硬性篩除類型。</x:v>
+      </x:c>
+      <x:c r="AA10"/>
+      <x:c r="AB10"/>
+      <x:c r="AC10"/>
+      <x:c r="AD10"/>
+      <x:c r="AE10"/>
+      <x:c r="AF10"/>
+      <x:c r="AG10"/>
+      <x:c r="AH10"/>
+      <x:c r="AI10"/>
+      <x:c r="AJ10"/>
+      <x:c r="AK10"/>
+      <x:c r="AL10"/>
+      <x:c r="AM10"/>
+    </x:row>
+    <x:row r="11" ht="54" customHeight="1">
+      <x:c r="A11" t="n">
+        <x:v>196</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>西华</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>最南抵西华，以已从五面峰瞰视，遂不复登。</x:v>
+      </x:c>
+      <x:c r="H11"/>
+      <x:c r="I11"/>
+      <x:c r="J11"/>
+      <x:c r="K11" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L11" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M11" t="str">
+        <x:v>作者明確抵達西華山，為具名山岳。</x:v>
+      </x:c>
+      <x:c r="AA11"/>
+      <x:c r="AB11"/>
+      <x:c r="AC11"/>
+      <x:c r="AD11"/>
+      <x:c r="AE11"/>
+      <x:c r="AF11"/>
+      <x:c r="AG11"/>
+      <x:c r="AH11"/>
+      <x:c r="AI11"/>
+      <x:c r="AJ11"/>
+      <x:c r="AK11"/>
+      <x:c r="AL11"/>
+      <x:c r="AM11"/>
+    </x:row>
+    <x:row r="12" ht="54" customHeight="1">
+      <x:c r="A12" t="n">
+        <x:v>197</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>一线天</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>峽谷</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>仍转出一线天，北逾一岭，二里，转而东，入小隐岩。</x:v>
+      </x:c>
+      <x:c r="H12" t="str">
+        <x:v>《弋阳县志》卷首〈龟峰图说〉｜識典古籍｜https://www.shidianguji.com/book/NLG312001072192/chapter/1ll4vbz35hwky</x:v>
+      </x:c>
+      <x:c r="I12" t="str">
+        <x:v>自此逾岭，双崖中裂，曰一线天。</x:v>
+      </x:c>
+      <x:c r="J12"/>
+      <x:c r="K12" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L12" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M12" t="str">
+        <x:v>一線天為作者再次經過的具名景觀，親身抵達，非硬性篩除類型。</x:v>
+      </x:c>
+      <x:c r="AA12"/>
+      <x:c r="AB12"/>
+      <x:c r="AC12"/>
+      <x:c r="AD12"/>
+      <x:c r="AE12"/>
+      <x:c r="AF12"/>
+      <x:c r="AG12"/>
+      <x:c r="AH12"/>
+      <x:c r="AI12"/>
+      <x:c r="AJ12"/>
+      <x:c r="AK12"/>
+      <x:c r="AL12"/>
+      <x:c r="AM12"/>
+    </x:row>
+    <x:row r="13" ht="54" customHeight="1">
+      <x:c r="A13" t="n">
+        <x:v>198</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>小隐岩</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>洞穴</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>仍转出一线天，北逾一岭，二里，转而东，入小隐岩。</x:v>
+      </x:c>
+      <x:c r="H13"/>
+      <x:c r="I13"/>
+      <x:c r="J13"/>
+      <x:c r="K13" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="L13" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="M13" t="str">
+        <x:v>作者進入小隱岩，為具名岩洞，具文化意義但定位待核。</x:v>
+      </x:c>
+      <x:c r="AA13"/>
+      <x:c r="AB13"/>
+      <x:c r="AC13"/>
+      <x:c r="AD13"/>
+      <x:c r="AE13"/>
+      <x:c r="AF13"/>
+      <x:c r="AG13"/>
+      <x:c r="AH13"/>
+      <x:c r="AI13"/>
+      <x:c r="AJ13"/>
+      <x:c r="AK13"/>
+      <x:c r="AL13"/>
+      <x:c r="AM13"/>
+    </x:row>
+    <x:row r="14" ht="54" customHeight="1">
+      <x:c r="A14" t="n">
+        <x:v>203</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>罗塘</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>聚落</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>聚落</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>遂由罗塘之大道，过一岭，始北转入山，竹树深蒨岩石高穹；但为释人架屋叠墙，无复本来面目，且知其非徐岩也。</x:v>
+      </x:c>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
+      <x:c r="K14" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L14" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M14" t="str">
+        <x:v>羅塘為作者途經之聚落，為穩定地名。</x:v>
+      </x:c>
+      <x:c r="AA14"/>
+      <x:c r="AB14"/>
+      <x:c r="AC14"/>
+      <x:c r="AD14"/>
+      <x:c r="AE14"/>
+      <x:c r="AF14"/>
+      <x:c r="AG14"/>
+      <x:c r="AH14"/>
+      <x:c r="AI14"/>
+      <x:c r="AJ14"/>
+      <x:c r="AK14"/>
+      <x:c r="AL14"/>
+      <x:c r="AM14"/>
+    </x:row>
+    <x:row r="15" ht="54" customHeight="1">
+      <x:c r="A15" t="n">
+        <x:v>206</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>象山</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>从其西二里，将抵象山，问所云徐岩，终不可得。</x:v>
+      </x:c>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
+      <x:c r="K15" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L15" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M15" t="str">
+        <x:v>象山為作者前往之具名山岳。</x:v>
+      </x:c>
+      <x:c r="AA15"/>
+      <x:c r="AB15"/>
+      <x:c r="AC15"/>
+      <x:c r="AD15"/>
+      <x:c r="AE15"/>
+      <x:c r="AF15"/>
+      <x:c r="AG15"/>
+      <x:c r="AH15"/>
+      <x:c r="AI15"/>
+      <x:c r="AJ15"/>
+      <x:c r="AK15"/>
+      <x:c r="AL15"/>
+      <x:c r="AM15"/>
+    </x:row>
+    <x:row r="16" ht="54" customHeight="1">
+      <x:c r="A16" t="n">
+        <x:v>212</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>朝真宫</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>宗教文化</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>寺廟／宮觀</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>二僧俱新至托宿，问之，亦不知其为徐岩与否，当即所称朝真宫矣。</x:v>
+      </x:c>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
+      <x:c r="K16" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="L16" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="M16" t="str">
+        <x:v>作者托宿之朝真宮，為具名宮觀，定位待核。</x:v>
+      </x:c>
+      <x:c r="AA16"/>
+      <x:c r="AB16"/>
+      <x:c r="AC16"/>
+      <x:c r="AD16"/>
+      <x:c r="AE16"/>
+      <x:c r="AF16"/>
+      <x:c r="AG16"/>
+      <x:c r="AH16"/>
+      <x:c r="AI16"/>
+      <x:c r="AJ16"/>
+      <x:c r="AK16"/>
+      <x:c r="AL16"/>
+      <x:c r="AM16"/>
+    </x:row>
+    <x:row r="17" ht="54" customHeight="1">
+      <x:c r="A17" t="n">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>象山</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>从暗中出，复西而南寻象山，其地虽暗而路可循，两崖前突，中坞不深而峻，当其中有坊峙焉。</x:v>
+      </x:c>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
+      <x:c r="K17" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L17" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M17" t="str">
+        <x:v>象山為作者尋找並抵達之具名山岳。</x:v>
+      </x:c>
+      <x:c r="AA17"/>
+      <x:c r="AB17"/>
+      <x:c r="AC17"/>
+      <x:c r="AD17"/>
+      <x:c r="AE17"/>
+      <x:c r="AF17"/>
+      <x:c r="AG17"/>
+      <x:c r="AH17"/>
+      <x:c r="AI17"/>
+      <x:c r="AJ17"/>
+      <x:c r="AK17"/>
+      <x:c r="AL17"/>
+      <x:c r="AM17"/>
+    </x:row>
+    <x:row r="18" ht="54" customHeight="1">
+      <x:c r="A18" t="n">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>曹山</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>饭而别观心，出曹山，而雨丝丝下。</x:v>
+      </x:c>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
+      <x:c r="K18" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L18" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M18" t="str">
+        <x:v>作者明確離開曹山，為實際身處地點</x:v>
+      </x:c>
+      <x:c r="AA18"/>
+      <x:c r="AB18"/>
+      <x:c r="AC18"/>
+      <x:c r="AD18"/>
+      <x:c r="AE18"/>
+      <x:c r="AF18"/>
+      <x:c r="AG18"/>
+      <x:c r="AH18"/>
+      <x:c r="AI18"/>
+      <x:c r="AJ18"/>
+      <x:c r="AK18"/>
+      <x:c r="AL18"/>
+      <x:c r="AM18"/>
+    </x:row>
+    <x:row r="19" ht="54" customHeight="1">
+      <x:c r="A19" t="n">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>崇仁</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
         <x:v>行政區</x:v>
       </x:c>
-      <x:c r="E8" s="59" t="str">
-        <x:v>城市／城</x:v>
-      </x:c>
-      <x:c r="F8" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G8" s="59" t="str">
-        <x:v>晨起，渡大溪之北，复西向行，八里，将至贵溪城，忽见溪南一桥门架空，以为城门与卷梁皆无此高跨之理。</x:v>
-      </x:c>
-      <x:c r="H8" s="59"/>
-      <x:c r="I8" s="59"/>
-      <x:c r="J8" s="59"/>
-      <x:c r="K8" s="59" t="str">
+      <x:c r="E19" t="str">
+        <x:v>縣</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>盖溪自曹山后岭北山峡而来，南下而转至鹏风桥者，此流尚细，而宜黄、崇仁之界，因逾接龙桥而西，即为崇之东南境。</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>《崇仁县志》卷一〈提封志〉｜識典古籍｜https://www.shidianguji.com/book/NA02851/chapter/1m6jjz17v2qzn</x:v>
+      </x:c>
+      <x:c r="I19" t="str">
+        <x:v>其东及东北为临川，其南及东南为宜黄，其西及西南为乐安，其北及西北为丰城。</x:v>
+      </x:c>
+      <x:c r="J19"/>
+      <x:c r="K19" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L8" s="59" t="str">
+      <x:c r="L19" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M8" s="59" t="str">
-        <x:v>貴溪城為縣城，作者將至，重要節點。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="59" t="n">
-        <x:v>185</x:v>
-      </x:c>
-      <x:c r="B9" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C9" s="59" t="str">
-        <x:v>张真人墓</x:v>
-      </x:c>
-      <x:c r="D9" s="59" t="str">
-        <x:v>歷史遺址</x:v>
-      </x:c>
-      <x:c r="E9" s="59" t="str">
-        <x:v>墓葬／陵墓</x:v>
-      </x:c>
-      <x:c r="F9" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G9" s="59" t="str">
-        <x:v>于是南经张真人墓。</x:v>
-      </x:c>
-      <x:c r="H9" s="59"/>
-      <x:c r="I9" s="59"/>
-      <x:c r="J9" s="59"/>
-      <x:c r="K9" s="59" t="str">
+      <x:c r="M19" t="str">
+        <x:v>作者明確進入崇仁縣境，為行政區劃</x:v>
+      </x:c>
+      <x:c r="AA19"/>
+      <x:c r="AB19"/>
+      <x:c r="AC19"/>
+      <x:c r="AD19"/>
+      <x:c r="AE19"/>
+      <x:c r="AF19"/>
+      <x:c r="AG19"/>
+      <x:c r="AH19"/>
+      <x:c r="AI19"/>
+      <x:c r="AJ19"/>
+      <x:c r="AK19"/>
+      <x:c r="AL19"/>
+      <x:c r="AM19"/>
+    </x:row>
+    <x:row r="20" ht="54" customHeight="1">
+      <x:c r="A20" t="n">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>大霍岭</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>自然地理</x:v>
+      </x:c>
+      <x:c r="E20" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F20" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G20" t="str">
+        <x:v>从此入山共三里，逾大霍岭，直逼龙骨山下。</x:v>
+      </x:c>
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
+      <x:c r="K20" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L9" s="59" t="str">
+      <x:c r="L20" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M9" s="59" t="str">
-        <x:v>作者實際經過之墓葬（張真人墓），為具名地標</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="54" customHeight="1">
-      <x:c r="A10" s="59" t="n">
-        <x:v>186</x:v>
-      </x:c>
-      <x:c r="B10" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C10" s="59" t="str">
-        <x:v>五面峰</x:v>
-      </x:c>
-      <x:c r="D10" s="59" t="str">
+      <x:c r="M20" t="str">
+        <x:v>作者翻越大霍嶺，為具名山嶺</x:v>
+      </x:c>
+      <x:c r="AA20"/>
+      <x:c r="AB20"/>
+      <x:c r="AC20"/>
+      <x:c r="AD20"/>
+      <x:c r="AE20"/>
+      <x:c r="AF20"/>
+      <x:c r="AG20"/>
+      <x:c r="AH20"/>
+      <x:c r="AI20"/>
+      <x:c r="AJ20"/>
+      <x:c r="AK20"/>
+      <x:c r="AL20"/>
+      <x:c r="AM20"/>
+    </x:row>
+    <x:row r="21" ht="54" customHeight="1">
+      <x:c r="A21" t="n">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="B21" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>龙骨山</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
         <x:v>自然地理</x:v>
       </x:c>
-      <x:c r="E10" s="59" t="str">
-        <x:v>山峰</x:v>
-      </x:c>
-      <x:c r="F10" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G10" s="59" t="str">
-        <x:v>溪流直逼五面峰下。</x:v>
-      </x:c>
-      <x:c r="H10" s="59"/>
-      <x:c r="I10" s="59"/>
-      <x:c r="J10" s="59"/>
-      <x:c r="K10" s="59" t="str">
+      <x:c r="E21" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F21" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G21" t="str">
+        <x:v>从此入山共三里，逾大霍岭，直逼龙骨山下。</x:v>
+      </x:c>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
+      <x:c r="K21" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L10" s="59" t="str">
+      <x:c r="L21" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M10" s="59" t="str">
-        <x:v>作者實際抵達之山峰，為穩定地理實體</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="54" customHeight="1">
-      <x:c r="A11" s="59" t="n">
-        <x:v>190</x:v>
-      </x:c>
-      <x:c r="B11" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C11" s="59" t="str">
-        <x:v>一线天</x:v>
-      </x:c>
-      <x:c r="D11" s="59" t="str">
+      <x:c r="M21" t="str">
+        <x:v>作者直逼龍骨山下，為具名山岳</x:v>
+      </x:c>
+      <x:c r="AA21"/>
+      <x:c r="AB21"/>
+      <x:c r="AC21"/>
+      <x:c r="AD21"/>
+      <x:c r="AE21"/>
+      <x:c r="AF21"/>
+      <x:c r="AG21"/>
+      <x:c r="AH21"/>
+      <x:c r="AI21"/>
+      <x:c r="AJ21"/>
+      <x:c r="AK21"/>
+      <x:c r="AL21"/>
+      <x:c r="AM21"/>
+    </x:row>
+    <x:row r="22" ht="54" customHeight="1">
+      <x:c r="A22" t="n">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>骨岭</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
         <x:v>自然地理</x:v>
       </x:c>
-      <x:c r="E11" s="59" t="str">
-        <x:v>峽谷</x:v>
-      </x:c>
-      <x:c r="F11" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G11" s="59" t="str">
-        <x:v>余意南下者为一线天，西上者为五面峰也。</x:v>
-      </x:c>
-      <x:c r="H11" s="59" t="str">
-        <x:v>《弋阳县志》卷首〈龟峰图说〉｜識典古籍｜https://www.shidianguji.com/book/NLG312001072192/chapter/1ll4vbz35hwky</x:v>
-      </x:c>
-      <x:c r="I11" s="59" t="str">
-        <x:v>自此逾岭，双崖中裂，曰一线天。</x:v>
-      </x:c>
-      <x:c r="J11" s="59"/>
-      <x:c r="K11" s="59" t="str">
+      <x:c r="E22" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>又二里，逾骨岭，水犹东注。</x:v>
+      </x:c>
+      <x:c r="H22"/>
+      <x:c r="I22"/>
+      <x:c r="J22"/>
+      <x:c r="K22" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L11" s="59" t="str">
+      <x:c r="L22" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M11" s="59" t="str">
-        <x:v>作者實際遊覽之一線天，為重要自然景觀</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="54" customHeight="1">
-      <x:c r="A12" s="59" t="n">
-        <x:v>191</x:v>
-      </x:c>
-      <x:c r="B12" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C12" s="59" t="str">
-        <x:v>五面峰</x:v>
-      </x:c>
-      <x:c r="D12" s="59" t="str">
+      <x:c r="M22" t="str">
+        <x:v>作者翻越骨嶺，為具名山嶺</x:v>
+      </x:c>
+      <x:c r="AA22"/>
+      <x:c r="AB22"/>
+      <x:c r="AC22"/>
+      <x:c r="AD22"/>
+      <x:c r="AE22"/>
+      <x:c r="AF22"/>
+      <x:c r="AG22"/>
+      <x:c r="AH22"/>
+      <x:c r="AI22"/>
+      <x:c r="AJ22"/>
+      <x:c r="AK22"/>
+      <x:c r="AL22"/>
+      <x:c r="AM22"/>
+    </x:row>
+    <x:row r="23" ht="54" customHeight="1">
+      <x:c r="A23" t="n">
+        <x:v>629</x:v>
+      </x:c>
+      <x:c r="B23" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>幞头岭</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
         <x:v>自然地理</x:v>
       </x:c>
-      <x:c r="E12" s="59" t="str">
-        <x:v>山峰</x:v>
-      </x:c>
-      <x:c r="F12" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G12" s="59" t="str">
-        <x:v>余意南下者为一线天，西上者为五面峰也。</x:v>
-      </x:c>
-      <x:c r="H12" s="59"/>
-      <x:c r="I12" s="59"/>
-      <x:c r="J12" s="59"/>
-      <x:c r="K12" s="59" t="str">
+      <x:c r="E23" t="str">
+        <x:v>山岳</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G23" t="str">
+        <x:v>又三里，下幞头岭，水始西流。</x:v>
+      </x:c>
+      <x:c r="H23"/>
+      <x:c r="I23"/>
+      <x:c r="J23"/>
+      <x:c r="K23" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L12" s="59" t="str">
+      <x:c r="L23" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M12" s="59" t="str">
-        <x:v>作者實際攀登之五面峰，為穩定地理實體</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="54" customHeight="1">
-      <x:c r="A13" s="59" t="n">
-        <x:v>192</x:v>
-      </x:c>
-      <x:c r="B13" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C13" s="59" t="str">
-        <x:v>西华</x:v>
-      </x:c>
-      <x:c r="D13" s="59" t="str">
+      <x:c r="M23" t="str">
+        <x:v>作者下幞頭嶺，為具名山嶺</x:v>
+      </x:c>
+      <x:c r="AA23"/>
+      <x:c r="AB23"/>
+      <x:c r="AC23"/>
+      <x:c r="AD23"/>
+      <x:c r="AE23"/>
+      <x:c r="AF23"/>
+      <x:c r="AG23"/>
+      <x:c r="AH23"/>
+      <x:c r="AI23"/>
+      <x:c r="AJ23"/>
+      <x:c r="AK23"/>
+      <x:c r="AL23"/>
+      <x:c r="AM23"/>
+    </x:row>
+    <x:row r="24" ht="54" customHeight="1">
+      <x:c r="A24" t="n">
+        <x:v>630</x:v>
+      </x:c>
+      <x:c r="B24" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>纯乡</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>聚落</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>聚落</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G24" t="str">
+        <x:v>又四里至纯乡，则一溪自南而北矣。</x:v>
+      </x:c>
+      <x:c r="H24"/>
+      <x:c r="I24"/>
+      <x:c r="J24"/>
+      <x:c r="K24" t="str">
+        <x:v>core</x:v>
+      </x:c>
+      <x:c r="L24" t="str">
+        <x:v>retain</x:v>
+      </x:c>
+      <x:c r="M24" t="str">
+        <x:v>作者抵達純鄉，為具名聚落</x:v>
+      </x:c>
+      <x:c r="AA24"/>
+      <x:c r="AB24"/>
+      <x:c r="AC24"/>
+      <x:c r="AD24"/>
+      <x:c r="AE24"/>
+      <x:c r="AF24"/>
+      <x:c r="AG24"/>
+      <x:c r="AH24"/>
+      <x:c r="AI24"/>
+      <x:c r="AJ24"/>
+      <x:c r="AK24"/>
+      <x:c r="AL24"/>
+      <x:c r="AM24"/>
+    </x:row>
+    <x:row r="25" ht="54" customHeight="1">
+      <x:c r="A25" t="n">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>纯乡村</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>村莊</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>村莊／寨</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G25" t="str">
+        <x:v>渡溪桥是为纯乡村，有居民颇众。</x:v>
+      </x:c>
+      <x:c r="H25"/>
+      <x:c r="I25"/>
+      <x:c r="J25"/>
+      <x:c r="K25" t="str">
+        <x:v>pending</x:v>
+      </x:c>
+      <x:c r="L25" t="str">
+        <x:v>review</x:v>
+      </x:c>
+      <x:c r="M25" t="str">
+        <x:v>作者描述純鄉村，為具名村莊；外部唯一對應未核</x:v>
+      </x:c>
+      <x:c r="AA25"/>
+      <x:c r="AB25"/>
+      <x:c r="AC25"/>
+      <x:c r="AD25"/>
+      <x:c r="AE25"/>
+      <x:c r="AF25"/>
+      <x:c r="AG25"/>
+      <x:c r="AH25"/>
+      <x:c r="AI25"/>
+      <x:c r="AJ25"/>
+      <x:c r="AK25"/>
+      <x:c r="AL25"/>
+      <x:c r="AM25"/>
+    </x:row>
+    <x:row r="26" ht="54" customHeight="1">
+      <x:c r="A26" t="n">
+        <x:v>633</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>干冈岭</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
         <x:v>自然地理</x:v>
       </x:c>
-      <x:c r="E13" s="59" t="str">
+      <x:c r="E26" t="str">
         <x:v>山岳</x:v>
       </x:c>
-      <x:c r="F13" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G13" s="59" t="str">
-        <x:v>先跻峰，攀磴里许而至绝顶，则南瞰西华，东瞰夹壁，西瞰南溪，北瞰城邑，皆在指顾。</x:v>
-      </x:c>
-      <x:c r="H13" s="59"/>
-      <x:c r="I13" s="59"/>
-      <x:c r="J13" s="59"/>
-      <x:c r="K13" s="59" t="str">
+      <x:c r="F26" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G26" t="str">
+        <x:v>南循小水一里，西登干冈岭，岭颇峻，逾岭而下，纯西南行矣。</x:v>
+      </x:c>
+      <x:c r="H26"/>
+      <x:c r="I26"/>
+      <x:c r="J26"/>
+      <x:c r="K26" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L13" s="59" t="str">
+      <x:c r="L26" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M13" s="59" t="str">
-        <x:v>作者實際眺望之西華山，為穩定地理實體</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="54" customHeight="1">
-      <x:c r="A14" s="59" t="n">
-        <x:v>195</x:v>
-      </x:c>
-      <x:c r="B14" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C14" s="59" t="str">
-        <x:v>一线天</x:v>
-      </x:c>
-      <x:c r="D14" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E14" s="59" t="str">
-        <x:v>峽谷</x:v>
-      </x:c>
-      <x:c r="F14" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G14" s="59" t="str">
-        <x:v>复从前磴南下一线天，则两崖并夹而上，直南即从峰顶下剖者，是为直峡。</x:v>
-      </x:c>
-      <x:c r="H14" s="59" t="str">
-        <x:v>《弋阳县志》卷首〈龟峰图说〉｜識典古籍｜https://www.shidianguji.com/book/NLG312001072192/chapter/1ll4vbz35hwky</x:v>
-      </x:c>
-      <x:c r="I14" s="59" t="str">
-        <x:v>自此逾岭，双崖中裂，曰一线天。</x:v>
-      </x:c>
-      <x:c r="J14" s="59"/>
-      <x:c r="K14" s="59" t="str">
+      <x:c r="M26" t="str">
+        <x:v>作者登越干岡嶺，為具名山嶺</x:v>
+      </x:c>
+      <x:c r="AA26"/>
+      <x:c r="AB26"/>
+      <x:c r="AC26"/>
+      <x:c r="AD26"/>
+      <x:c r="AE26"/>
+      <x:c r="AF26"/>
+      <x:c r="AG26"/>
+      <x:c r="AH26"/>
+      <x:c r="AI26"/>
+      <x:c r="AJ26"/>
+      <x:c r="AK26"/>
+      <x:c r="AL26"/>
+      <x:c r="AM26"/>
+    </x:row>
+    <x:row r="27" ht="54" customHeight="1">
+      <x:c r="A27" t="n">
+        <x:v>636</x:v>
+      </x:c>
+      <x:c r="B27" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>巴溪</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>水系</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>江河</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G27" t="str">
+        <x:v>又西五里，过练树桥，桥跨巴溪之上。</x:v>
+      </x:c>
+      <x:c r="H27"/>
+      <x:c r="I27"/>
+      <x:c r="J27"/>
+      <x:c r="K27" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L14" s="59" t="str">
+      <x:c r="L27" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M14" s="59" t="str">
-        <x:v>一線天為作者親身經過的具名峽谷或岩隙景觀，屬地理實體，非硬性篩除類型。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="54" customHeight="1">
-      <x:c r="A15" s="59" t="n">
-        <x:v>196</x:v>
-      </x:c>
-      <x:c r="B15" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C15" s="59" t="str">
-        <x:v>西华</x:v>
-      </x:c>
-      <x:c r="D15" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E15" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F15" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G15" s="59" t="str">
-        <x:v>最南抵西华，以已从五面峰瞰视，遂不复登。</x:v>
-      </x:c>
-      <x:c r="H15" s="59"/>
-      <x:c r="I15" s="59"/>
-      <x:c r="J15" s="59"/>
-      <x:c r="K15" s="59" t="str">
+      <x:c r="M27" t="str">
+        <x:v>巴溪為具名河流，作者經過其橋</x:v>
+      </x:c>
+      <x:c r="AA27"/>
+      <x:c r="AB27"/>
+      <x:c r="AC27"/>
+      <x:c r="AD27"/>
+      <x:c r="AE27"/>
+      <x:c r="AF27"/>
+      <x:c r="AG27"/>
+      <x:c r="AH27"/>
+      <x:c r="AI27"/>
+      <x:c r="AJ27"/>
+      <x:c r="AK27"/>
+      <x:c r="AL27"/>
+      <x:c r="AM27"/>
+    </x:row>
+    <x:row r="28" ht="54" customHeight="1">
+      <x:c r="A28" t="n">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="B28" t="str">
+        <x:v>二十三日</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
+        <x:v>朱碧街</x:v>
+      </x:c>
+      <x:c r="D28" t="str">
+        <x:v>聚落</x:v>
+      </x:c>
+      <x:c r="E28" t="str">
+        <x:v>聚落</x:v>
+      </x:c>
+      <x:c r="F28" t="str">
+        <x:v>經過</x:v>
+      </x:c>
+      <x:c r="G28" t="str">
+        <x:v>自练树桥又五里而至朱碧街。</x:v>
+      </x:c>
+      <x:c r="H28"/>
+      <x:c r="I28"/>
+      <x:c r="J28"/>
+      <x:c r="K28" t="str">
         <x:v>core</x:v>
       </x:c>
-      <x:c r="L15" s="59" t="str">
+      <x:c r="L28" t="str">
         <x:v>retain</x:v>
       </x:c>
-      <x:c r="M15" s="59" t="str">
-        <x:v>作者明確抵達西華山，為具名山岳。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="54" customHeight="1">
-      <x:c r="A16" s="59" t="n">
-        <x:v>197</x:v>
-      </x:c>
-      <x:c r="B16" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C16" s="59" t="str">
-        <x:v>一线天</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>峽谷</x:v>
-      </x:c>
-      <x:c r="F16" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G16" s="59" t="str">
-        <x:v>仍转出一线天，北逾一岭，二里，转而东，入小隐岩。</x:v>
-      </x:c>
-      <x:c r="H16" s="59" t="str">
-        <x:v>《弋阳县志》卷首〈龟峰图说〉｜識典古籍｜https://www.shidianguji.com/book/NLG312001072192/chapter/1ll4vbz35hwky</x:v>
-      </x:c>
-      <x:c r="I16" s="59" t="str">
-        <x:v>自此逾岭，双崖中裂，曰一线天。</x:v>
-      </x:c>
-      <x:c r="J16" s="59"/>
-      <x:c r="K16" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L16" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M16" s="59" t="str">
-        <x:v>一線天為作者再次經過的具名景觀，親身抵達，非硬性篩除類型。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="54" customHeight="1">
-      <x:c r="A17" s="59" t="n">
-        <x:v>198</x:v>
-      </x:c>
-      <x:c r="B17" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C17" s="59" t="str">
-        <x:v>小隐岩</x:v>
-      </x:c>
-      <x:c r="D17" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E17" s="59" t="str">
-        <x:v>洞穴</x:v>
-      </x:c>
-      <x:c r="F17" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G17" s="59" t="str">
-        <x:v>仍转出一线天，北逾一岭，二里，转而东，入小隐岩。</x:v>
-      </x:c>
-      <x:c r="H17" s="59"/>
-      <x:c r="I17" s="59"/>
-      <x:c r="J17" s="59"/>
-      <x:c r="K17" s="59" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="L17" s="59" t="str">
-        <x:v>review</x:v>
-      </x:c>
-      <x:c r="M17" s="59" t="str">
-        <x:v>作者進入小隱岩，為具名岩洞，具文化意義但定位待核。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="54" customHeight="1">
-      <x:c r="A18" s="59" t="n">
-        <x:v>203</x:v>
-      </x:c>
-      <x:c r="B18" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C18" s="59" t="str">
-        <x:v>罗塘</x:v>
-      </x:c>
-      <x:c r="D18" s="59" t="str">
-        <x:v>聚落</x:v>
-      </x:c>
-      <x:c r="E18" s="59" t="str">
-        <x:v>聚落</x:v>
-      </x:c>
-      <x:c r="F18" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G18" s="59" t="str">
-        <x:v>遂由罗塘之大道，过一岭，始北转入山，竹树深蒨岩石高穹；但为释人架屋叠墙，无复本来面目，且知其非徐岩也。</x:v>
-      </x:c>
-      <x:c r="H18" s="59"/>
-      <x:c r="I18" s="59"/>
-      <x:c r="J18" s="59"/>
-      <x:c r="K18" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L18" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M18" s="59" t="str">
-        <x:v>羅塘為作者途經之聚落，為穩定地名。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="54" customHeight="1">
-      <x:c r="A19" s="59" t="n">
-        <x:v>206</x:v>
-      </x:c>
-      <x:c r="B19" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C19" s="59" t="str">
-        <x:v>象山</x:v>
-      </x:c>
-      <x:c r="D19" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E19" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F19" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G19" s="59" t="str">
-        <x:v>从其西二里，将抵象山，问所云徐岩，终不可得。</x:v>
-      </x:c>
-      <x:c r="H19" s="59"/>
-      <x:c r="I19" s="59"/>
-      <x:c r="J19" s="59"/>
-      <x:c r="K19" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L19" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M19" s="59" t="str">
-        <x:v>象山為作者前往之具名山岳。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="54" customHeight="1">
-      <x:c r="A20" s="59" t="n">
-        <x:v>212</x:v>
-      </x:c>
-      <x:c r="B20" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C20" s="59" t="str">
-        <x:v>朝真宫</x:v>
-      </x:c>
-      <x:c r="D20" s="59" t="str">
-        <x:v>宗教文化</x:v>
-      </x:c>
-      <x:c r="E20" s="59" t="str">
-        <x:v>寺廟／宮觀</x:v>
-      </x:c>
-      <x:c r="F20" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G20" s="59" t="str">
-        <x:v>二僧俱新至托宿，问之，亦不知其为徐岩与否，当即所称朝真宫矣。</x:v>
-      </x:c>
-      <x:c r="H20" s="59"/>
-      <x:c r="I20" s="59"/>
-      <x:c r="J20" s="59"/>
-      <x:c r="K20" s="59" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="L20" s="59" t="str">
-        <x:v>review</x:v>
-      </x:c>
-      <x:c r="M20" s="59" t="str">
-        <x:v>作者托宿之朝真宮，為具名宮觀，定位待核。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="54" customHeight="1">
-      <x:c r="A21" s="59" t="n">
-        <x:v>213</x:v>
-      </x:c>
-      <x:c r="B21" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C21" s="59" t="str">
-        <x:v>象山</x:v>
-      </x:c>
-      <x:c r="D21" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E21" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F21" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G21" s="59" t="str">
-        <x:v>从暗中出，复西而南寻象山，其地虽暗而路可循，两崖前突，中坞不深而峻，当其中有坊峙焉。</x:v>
-      </x:c>
-      <x:c r="H21" s="59"/>
-      <x:c r="I21" s="59"/>
-      <x:c r="J21" s="59"/>
-      <x:c r="K21" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L21" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M21" s="59" t="str">
-        <x:v>象山為作者尋找並抵達之具名山岳。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="54" customHeight="1">
-      <x:c r="A22" s="59" t="n">
-        <x:v>620</x:v>
-      </x:c>
-      <x:c r="B22" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C22" s="59" t="str">
-        <x:v>曹山</x:v>
-      </x:c>
-      <x:c r="D22" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E22" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F22" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G22" s="59" t="str">
-        <x:v>饭而别观心，出曹山，而雨丝丝下。</x:v>
-      </x:c>
-      <x:c r="H22" s="59"/>
-      <x:c r="I22" s="59"/>
-      <x:c r="J22" s="59"/>
-      <x:c r="K22" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L22" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M22" s="59" t="str">
-        <x:v>作者明確離開曹山，為實際身處地點</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23" ht="54" customHeight="1">
-      <x:c r="A23" s="59" t="n">
-        <x:v>625</x:v>
-      </x:c>
-      <x:c r="B23" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C23" s="59" t="str">
-        <x:v>崇仁</x:v>
-      </x:c>
-      <x:c r="D23" s="59" t="str">
-        <x:v>行政區</x:v>
-      </x:c>
-      <x:c r="E23" s="59" t="str">
-        <x:v>縣</x:v>
-      </x:c>
-      <x:c r="F23" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G23" s="59" t="str">
-        <x:v>盖溪自曹山后岭北山峡而来，南下而转至鹏风桥者，此流尚细，而宜黄、崇仁之界，因逾接龙桥而西，即为崇之东南境。</x:v>
-      </x:c>
-      <x:c r="H23" s="59" t="str">
-        <x:v>《崇仁县志》卷一〈提封志〉｜識典古籍｜https://www.shidianguji.com/book/NA02851/chapter/1m6jjz17v2qzn</x:v>
-      </x:c>
-      <x:c r="I23" s="59" t="str">
-        <x:v>其东及东北为临川，其南及东南为宜黄，其西及西南为乐安，其北及西北为丰城。</x:v>
-      </x:c>
-      <x:c r="J23" s="59"/>
-      <x:c r="K23" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L23" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M23" s="59" t="str">
-        <x:v>作者明確進入崇仁縣境，為行政區劃</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24" ht="54" customHeight="1">
-      <x:c r="A24" s="59" t="n">
-        <x:v>626</x:v>
-      </x:c>
-      <x:c r="B24" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C24" s="59" t="str">
-        <x:v>大霍岭</x:v>
-      </x:c>
-      <x:c r="D24" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E24" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F24" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G24" s="59" t="str">
-        <x:v>从此入山共三里，逾大霍岭，直逼龙骨山下。</x:v>
-      </x:c>
-      <x:c r="H24" s="59"/>
-      <x:c r="I24" s="59"/>
-      <x:c r="J24" s="59"/>
-      <x:c r="K24" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L24" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M24" s="59" t="str">
-        <x:v>作者翻越大霍嶺，為具名山嶺</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="54" customHeight="1">
-      <x:c r="A25" s="59" t="n">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="B25" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C25" s="59" t="str">
-        <x:v>龙骨山</x:v>
-      </x:c>
-      <x:c r="D25" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E25" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F25" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G25" s="59" t="str">
-        <x:v>从此入山共三里，逾大霍岭，直逼龙骨山下。</x:v>
-      </x:c>
-      <x:c r="H25" s="59"/>
-      <x:c r="I25" s="59"/>
-      <x:c r="J25" s="59"/>
-      <x:c r="K25" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L25" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M25" s="59" t="str">
-        <x:v>作者直逼龍骨山下，為具名山岳</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="54" customHeight="1">
-      <x:c r="A26" s="59" t="n">
-        <x:v>628</x:v>
-      </x:c>
-      <x:c r="B26" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C26" s="59" t="str">
-        <x:v>骨岭</x:v>
-      </x:c>
-      <x:c r="D26" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E26" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F26" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G26" s="59" t="str">
-        <x:v>又二里，逾骨岭，水犹东注。</x:v>
-      </x:c>
-      <x:c r="H26" s="59"/>
-      <x:c r="I26" s="59"/>
-      <x:c r="J26" s="59"/>
-      <x:c r="K26" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L26" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M26" s="59" t="str">
-        <x:v>作者翻越骨嶺，為具名山嶺</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27" ht="54" customHeight="1">
-      <x:c r="A27" s="59" t="n">
-        <x:v>629</x:v>
-      </x:c>
-      <x:c r="B27" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C27" s="59" t="str">
-        <x:v>幞头岭</x:v>
-      </x:c>
-      <x:c r="D27" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E27" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F27" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G27" s="59" t="str">
-        <x:v>又三里，下幞头岭，水始西流。</x:v>
-      </x:c>
-      <x:c r="H27" s="59"/>
-      <x:c r="I27" s="59"/>
-      <x:c r="J27" s="59"/>
-      <x:c r="K27" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L27" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M27" s="59" t="str">
-        <x:v>作者下幞頭嶺，為具名山嶺</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28" ht="54" customHeight="1">
-      <x:c r="A28" s="59" t="n">
-        <x:v>630</x:v>
-      </x:c>
-      <x:c r="B28" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C28" s="59" t="str">
-        <x:v>纯乡</x:v>
-      </x:c>
-      <x:c r="D28" s="59" t="str">
-        <x:v>聚落</x:v>
-      </x:c>
-      <x:c r="E28" s="59" t="str">
-        <x:v>聚落</x:v>
-      </x:c>
-      <x:c r="F28" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G28" s="59" t="str">
-        <x:v>又四里至纯乡，则一溪自南而北矣。</x:v>
-      </x:c>
-      <x:c r="H28" s="59"/>
-      <x:c r="I28" s="59"/>
-      <x:c r="J28" s="59"/>
-      <x:c r="K28" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L28" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M28" s="59" t="str">
-        <x:v>作者抵達純鄉，為具名聚落</x:v>
+      <x:c r="M28" t="str">
+        <x:v>作者明確從練樹橋行五里抵達朱碧街，為實際經過的聚落。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="54" customHeight="1">
-      <x:c r="A29" s="59" t="n">
-        <x:v>631</x:v>
-      </x:c>
-      <x:c r="B29" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C29" s="59" t="str">
-        <x:v>纯乡村</x:v>
-      </x:c>
-      <x:c r="D29" s="59" t="str">
-        <x:v>村莊</x:v>
-      </x:c>
-      <x:c r="E29" s="59" t="str">
-        <x:v>村莊／寨</x:v>
-      </x:c>
-      <x:c r="F29" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G29" s="59" t="str">
-        <x:v>渡溪桥是为纯乡村，有居民颇众。</x:v>
-      </x:c>
-      <x:c r="H29" s="59"/>
-      <x:c r="I29" s="59"/>
-      <x:c r="J29" s="59"/>
-      <x:c r="K29" s="59" t="str">
-        <x:v>pending</x:v>
-      </x:c>
-      <x:c r="L29" s="59" t="str">
-        <x:v>review</x:v>
-      </x:c>
-      <x:c r="M29" s="59" t="str">
-        <x:v>作者描述純鄉村，為具名村莊；外部唯一對應未核</x:v>
-      </x:c>
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
+      <x:c r="I29"/>
+      <x:c r="J29"/>
+      <x:c r="K29"/>
+      <x:c r="L29"/>
+      <x:c r="M29"/>
     </x:row>
     <x:row r="30" ht="54" customHeight="1">
-      <x:c r="A30" s="59" t="n">
-        <x:v>633</x:v>
-      </x:c>
-      <x:c r="B30" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C30" s="59" t="str">
-        <x:v>干冈岭</x:v>
-      </x:c>
-      <x:c r="D30" s="59" t="str">
-        <x:v>自然地理</x:v>
-      </x:c>
-      <x:c r="E30" s="59" t="str">
-        <x:v>山岳</x:v>
-      </x:c>
-      <x:c r="F30" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G30" s="59" t="str">
-        <x:v>南循小水一里，西登干冈岭，岭颇峻，逾岭而下，纯西南行矣。</x:v>
-      </x:c>
-      <x:c r="H30" s="59"/>
-      <x:c r="I30" s="59"/>
-      <x:c r="J30" s="59"/>
-      <x:c r="K30" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L30" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M30" s="59" t="str">
-        <x:v>作者登越干岡嶺，為具名山嶺</x:v>
-      </x:c>
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+      <x:c r="I30"/>
+      <x:c r="J30"/>
+      <x:c r="K30"/>
+      <x:c r="L30"/>
+      <x:c r="M30"/>
     </x:row>
     <x:row r="31" ht="54" customHeight="1">
-      <x:c r="A31" s="59" t="n">
-        <x:v>636</x:v>
-      </x:c>
-      <x:c r="B31" s="59" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C31" s="59" t="str">
-        <x:v>巴溪</x:v>
-      </x:c>
-      <x:c r="D31" s="59" t="str">
-        <x:v>水系</x:v>
-      </x:c>
-      <x:c r="E31" s="59" t="str">
-        <x:v>江河</x:v>
-      </x:c>
-      <x:c r="F31" s="59" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G31" s="59" t="str">
-        <x:v>又西五里，过练树桥，桥跨巴溪之上。</x:v>
-      </x:c>
-      <x:c r="H31" s="59"/>
-      <x:c r="I31" s="59"/>
-      <x:c r="J31" s="59"/>
-      <x:c r="K31" s="59" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L31" s="59" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M31" s="59" t="str">
-        <x:v>巴溪為具名河流，作者經過其橋</x:v>
-      </x:c>
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
+      <x:c r="I31"/>
+      <x:c r="J31"/>
+      <x:c r="K31"/>
+      <x:c r="L31"/>
+      <x:c r="M31"/>
     </x:row>
     <x:row r="32" ht="54" customHeight="1">
-      <x:c r="A32" s="32" t="n">
-        <x:v>650</x:v>
-      </x:c>
-      <x:c r="B32" s="32" t="str">
-        <x:v>二十三日</x:v>
-      </x:c>
-      <x:c r="C32" s="32" t="str">
-        <x:v>朱碧街</x:v>
-      </x:c>
-      <x:c r="D32" s="32" t="str">
-        <x:v>聚落</x:v>
-      </x:c>
-      <x:c r="E32" s="32" t="str">
-        <x:v>聚落</x:v>
-      </x:c>
-      <x:c r="F32" s="32" t="str">
-        <x:v>經過</x:v>
-      </x:c>
-      <x:c r="G32" s="32" t="str">
-        <x:v>自练树桥又五里而至朱碧街。</x:v>
-      </x:c>
-      <x:c r="H32" s="32"/>
-      <x:c r="I32" s="32"/>
-      <x:c r="J32" s="32"/>
-      <x:c r="K32" s="32" t="str">
-        <x:v>core</x:v>
-      </x:c>
-      <x:c r="L32" s="32" t="str">
-        <x:v>retain</x:v>
-      </x:c>
-      <x:c r="M32" s="32" t="str">
-        <x:v>作者明確從練樹橋行五里抵達朱碧街，為實際經過的聚落。</x:v>
-      </x:c>
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
+      <x:c r="G32"/>
+      <x:c r="H32"/>
+      <x:c r="I32"/>
+      <x:c r="J32"/>
+      <x:c r="K32"/>
+      <x:c r="L32"/>
+      <x:c r="M32"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:M1"/>
-    <x:mergeCell ref="A2:M2"/>
-    <x:mergeCell ref="A3:M3"/>
-    <x:mergeCell ref="A4:M4"/>
-    <x:mergeCell ref="A5:M5"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6b9a952089f4094"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a8bcd6482cc4345"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2529,7 +2871,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R94114b88c3304d7a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfe038d7ce104471"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>